<commit_message>
Batch add & roadmap update
</commit_message>
<xml_diff>
--- a/CPFR_VDS_CPH_Docs/TPM/CPH OP1.xlsx
+++ b/CPFR_VDS_CPH_Docs/TPM/CPH OP1.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29912"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://chewycomllc-my.sharepoint.com/personal/nnelson2_chewy_com/Documents/Outward Hound/Desktop/garb/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://chewycomllc-my.sharepoint.com/personal/nmiles1_chewy_com/Documents/Documents/GitHub/Hermes/CPFR_VDS_CPH_Docs/TPM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{5A12A9F2-6EE6-4835-A106-BB87129D9CA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{463F9132-6BF7-40C1-9BAF-29D70170B0D3}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{5A12A9F2-6EE6-4835-A106-BB87129D9CA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6C258D1A-D8FE-414A-B274-9A7BBD78E06C}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6FE411E3-C88D-4AEB-BC67-70065D362FD2}"/>
+    <workbookView xWindow="28680" yWindow="0" windowWidth="29040" windowHeight="15720" xr2:uid="{6FE411E3-C88D-4AEB-BC67-70065D362FD2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -101,15 +101,18 @@
     <t>P0</t>
   </si>
   <si>
+    <t>In-Stock (SCO/PMO): Dave Livesay</t>
+  </si>
+  <si>
     <t>New Process</t>
   </si>
   <si>
-    <t>In-Stock (SCO/PMO): Dave Livesay</t>
-  </si>
-  <si>
     <t xml:space="preserve">CPH Integration </t>
   </si>
   <si>
+    <t>Today, Chewy lacks a centralized and scalable platform for vendors to access the data required to effectively manage their supply chain and operational performance. Vendors rely on fragmented email communications, receiving up to 65 separate emails per month across EDI, Supply, Demand, In Stock, Operations, and Vendor Compliance, creating information overload, limited role based relevance, and reduced actionability. This model drives frustration, delayed response, and missed improvement opportunities, and cannot scale to support additional high value reporting without degrading the vendor experience. At the same time, across both CPFR and Vendor Compliance, CPH is a prerequisite to unlock and operationalize an estimated $12M in total annual entitlement, including chargeback expansion, operational efficiency gains, vendor enablement benefits, and broader enterprise alignment opportunities.To strengthen our competitive position, Chewy must elevate our vendor capabilities to align with industry benchmarks set by leaders such as Amazon and Walmart, whose Vendor Central and Luminate platforms deliver centralized reporting and analytics, role based access, and integrated performance management at scale. Without a centralized solution such as CPH, we are constrained in our ability to scale vendor accountability, improve compliance, enhance operational efficiency, and fully realize this financial and strategic value.</t>
+  </si>
+  <si>
     <t>Establish CPH as the centralized platform for CPFR and Vendor Compliance reporting, enabling structured program enrollment and controlled access at the vendor level. Through governed access controls, vendors would manage their own user permissions and role based distribution, ensuring the right stakeholders receive the right information. CPH would serve as the single source of truth for report access and historical visibility, creating a scalable foundation for expanded program deployment, improved transparency, and faster data driven decision making across the supply chain.</t>
   </si>
   <si>
@@ -125,13 +128,10 @@
     <t>1.) Vendor experience, 2.) Vendor analytics, action, and improvement, 3.) Infrastructure scalability and governance, 4.) Dispute resolution efficiency, 5.) Financial entitlement capture and accountability, 6.) Competitive parity with industry benchmarks (Amazon Vendor Central, Walmart Luminate)</t>
   </si>
   <si>
+    <t xml:space="preserve">$10M Chargeback Expansion, $600k Operation Efficiency, $712 Vendor Enablement, and  $375k Data Alignment and Accuracy </t>
+  </si>
+  <si>
     <t>Leadership Documents</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$10M Chargeback Expansion, $600k Operation Efficiency, $712 Vendor Enablement, and  $375k Data Alignment and Accuacy </t>
-  </si>
-  <si>
-    <t>Today, Chewy lacks a centralized and scalable platform for vendors to access the data required to effectively manage their supply chain and operational performance. Vendors rely on fragmented email communications, receiving up to 65 separate emails per month across EDI, Supply, Demand, In Stock, Operations, and Vendor Compliance, creating information overload, limited role based relevance, and reduced actionability. This model drives frustration, delayed response, and missed improvement opportunities, and cannot scale to support additional high value reporting without degrading the vendor experience. At the same time, across both CPFR and Vendor Compliance, CPH is a prerequisite to unlock and operationalize an estimated $12M in total annual entitlement, including chargeback expansion, operational efficiency gains, vendor enablement benefits, and broader enterprise alignment opportunities.To strengthen our competitive position, Chewy must elevate our vendor capabilities to align with industry benchmarks set by leaders such as Amazon and Walmart, whose Vendor Central and Luminate platforms deliver centralized reporting and analytics, role based access, and integrated performance management at scale. Without a centralized solution such as CPH, we are constrained in our ability to scale vendor accountability, improve compliance, enhance operational efficiency, and fully realize this financial and strategic value.</t>
   </si>
 </sst>
 </file>
@@ -141,7 +141,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -298,15 +298,86 @@
   </cellStyleXfs>
   <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -314,88 +385,17 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -733,7 +733,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F782C934-0EEB-410D-9BB1-D7149395A65A}">
   <dimension ref="A1:T3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.28515625" bestFit="1" customWidth="1"/>
@@ -753,142 +753,142 @@
     <col min="17" max="17" width="31.140625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="96.28515625" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="4.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="21.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:20">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6"/>
-      <c r="I1" s="5" t="s">
+      <c r="H1" s="1"/>
+      <c r="I1" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="7"/>
-      <c r="M1" s="5" t="s">
+      <c r="L1" s="2"/>
+      <c r="M1" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="N1" s="7"/>
-      <c r="O1" s="3" t="s">
+      <c r="N1" s="2"/>
+      <c r="O1" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="P1" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="Q1" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="R1" s="5" t="s">
+      <c r="R1" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="S1" s="7"/>
-      <c r="T1" s="2" t="s">
+      <c r="S1" s="2"/>
+      <c r="T1" s="20" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="8"/>
-      <c r="B2" s="9" t="s">
+    <row r="2" spans="1:20" ht="48.95" thickBot="1">
+      <c r="A2" s="19"/>
+      <c r="B2" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="9"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="15" t="s">
+      <c r="C2" s="21"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="M2" s="16"/>
-      <c r="N2" s="15" t="s">
+      <c r="M2" s="26"/>
+      <c r="N2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="O2" s="14"/>
-      <c r="P2" s="16"/>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="15" t="s">
+      <c r="O2" s="27"/>
+      <c r="P2" s="26"/>
+      <c r="Q2" s="17"/>
+      <c r="R2" s="17"/>
+      <c r="S2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="T2" s="9" t="s">
+      <c r="T2" s="21" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:20" s="27" customFormat="1" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="21">
+    <row r="3" spans="1:20" s="15" customFormat="1" ht="409.5" customHeight="1">
+      <c r="A3" s="9">
         <f t="shared" ref="A3" si="0">A2+1</f>
         <v>1</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="23" t="s">
+      <c r="F3" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" s="7"/>
+      <c r="I3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="K3" s="8"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="N3" s="7"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="R3" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="S3" s="5"/>
+      <c r="T3" s="14" t="s">
         <v>31</v>
-      </c>
-      <c r="G3" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="H3" s="19"/>
-      <c r="I3" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="J3" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="K3" s="20"/>
-      <c r="L3" s="17"/>
-      <c r="M3" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="N3" s="19"/>
-      <c r="O3" s="17"/>
-      <c r="P3" s="17"/>
-      <c r="Q3" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="R3" s="25" t="s">
-        <v>30</v>
-      </c>
-      <c r="S3" s="17"/>
-      <c r="T3" s="26" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -903,12 +903,12 @@
     <mergeCell ref="K1:K2"/>
     <mergeCell ref="M1:M2"/>
     <mergeCell ref="O1:O2"/>
+    <mergeCell ref="F1:F2"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="T3" r:id="rId1" display="https://chewycomllc.sharepoint.com/sites/VendorCompliance/_layouts/15/guestaccess.aspx?share=IgATcuMvww-1R4PjoGnqSg8qAR_SyoSSW1SJLThchmnsae4&amp;e=cd7euQ" xr:uid="{F449FB6B-B1F4-434A-A6F5-6A867615B793}"/>

</xml_diff>